<commit_message>
sync total local a web
</commit_message>
<xml_diff>
--- a/flujo_proyectado.xlsx
+++ b/flujo_proyectado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\manager8\comunes\importacion\api_cluster\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hrubilar\Recotoner Dropbox\henry rubilar\C_Henry_Rubilar\PROYECTO FLUJO DE CAJA\api_cluster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77CEA80-9897-4407-BCDA-347C63345436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45583762-F346-465D-A102-B53AA3B9C235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D4753735-02AC-4A26-9DB4-FFC87C45DC2E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
   <si>
     <t xml:space="preserve">1.01.05.01 - Facturas por cobrar Nacional- FLUJO </t>
   </si>
@@ -78,6 +78,15 @@
   </si>
   <si>
     <t>CLASIFICACION</t>
+  </si>
+  <si>
+    <t>TIPO DE MOVIMIENTO</t>
+  </si>
+  <si>
+    <t>INGRESO</t>
+  </si>
+  <si>
+    <t>EGRESO</t>
   </si>
 </sst>
 </file>
@@ -121,7 +130,7 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -458,588 +467,633 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B690EF9-61EE-464E-B377-DAD3AF0A4931}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="56.5546875" customWidth="1"/>
-    <col min="2" max="2" width="23" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="13" width="11.5546875" style="1"/>
+    <col min="2" max="2" width="23.109375" customWidth="1"/>
+    <col min="3" max="3" width="23" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.5546875" style="1"/>
+    <col min="7" max="7" width="11.5546875" style="3"/>
+    <col min="8" max="14" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="2">
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2">
         <v>45839</v>
       </c>
-      <c r="C1" s="2">
+      <c r="D1" s="2">
         <v>45870</v>
       </c>
-      <c r="D1" s="2">
+      <c r="E1" s="2">
         <v>45901</v>
       </c>
-      <c r="E1" s="2">
+      <c r="F1" s="2">
         <v>45931</v>
       </c>
-      <c r="F1" s="2">
+      <c r="G1" s="2">
         <v>45962</v>
       </c>
-      <c r="G1" s="2">
+      <c r="H1" s="2">
         <v>45992</v>
       </c>
-      <c r="H1" s="2">
+      <c r="I1" s="2">
         <v>46023</v>
       </c>
-      <c r="I1" s="2">
+      <c r="J1" s="2">
         <v>46054</v>
       </c>
-      <c r="J1" s="2">
+      <c r="K1" s="2">
         <v>46082</v>
       </c>
-      <c r="K1" s="2">
+      <c r="L1" s="2">
         <v>46113</v>
       </c>
-      <c r="L1" s="2">
+      <c r="M1" s="2">
         <v>46143</v>
       </c>
-      <c r="M1" s="2">
+      <c r="N1" s="2">
         <v>46174</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1">
         <f>39309118+3412482</f>
         <v>42721600</v>
       </c>
-      <c r="C2" s="3">
+      <c r="D2" s="1">
         <v>50854293.000000007</v>
       </c>
-      <c r="D2" s="3">
+      <c r="E2" s="1">
         <v>52178049</v>
       </c>
-      <c r="E2" s="3">
+      <c r="F2" s="1">
         <v>55266813</v>
       </c>
-      <c r="F2" s="3">
+      <c r="G2" s="3">
         <v>59679333.000000007</v>
       </c>
-      <c r="G2" s="3">
+      <c r="H2" s="1">
         <v>60341211</v>
       </c>
-      <c r="H2" s="3">
+      <c r="I2" s="1">
         <v>65305296</v>
       </c>
-      <c r="I2" s="3">
+      <c r="J2" s="1">
         <v>66518739</v>
       </c>
-      <c r="J2" s="3">
+      <c r="K2" s="1">
         <v>73137519</v>
       </c>
-      <c r="K2" s="3">
+      <c r="L2" s="1">
         <v>78763482</v>
       </c>
-      <c r="L2" s="3">
+      <c r="M2" s="1">
         <v>81741933</v>
       </c>
-      <c r="M2" s="3">
+      <c r="N2" s="1">
         <v>82624437</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1">
         <v>30000000</v>
       </c>
-      <c r="C3" s="3">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3">
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
         <v>0</v>
       </c>
       <c r="G3" s="3">
         <v>0</v>
       </c>
-      <c r="H3" s="3">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
-      <c r="J3" s="3">
-        <v>0</v>
-      </c>
-      <c r="K3" s="3">
-        <v>0</v>
-      </c>
-      <c r="L3" s="3">
-        <v>0</v>
-      </c>
-      <c r="M3" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="1">
         <v>9844270</v>
       </c>
-      <c r="C4" s="3">
+      <c r="D4" s="1">
         <v>4842222</v>
       </c>
-      <c r="D4" s="3">
+      <c r="E4" s="1">
         <v>4842222</v>
       </c>
-      <c r="E4" s="3">
-        <v>4842222</v>
-      </c>
-      <c r="F4" s="3">
+      <c r="F4" s="1">
         <v>4842222</v>
       </c>
       <c r="G4" s="3">
         <v>4842222</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="1">
         <v>4842222</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="1">
         <v>4842222</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="1">
         <v>4842222</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="1">
         <v>4842222</v>
       </c>
-      <c r="L4" s="3">
+      <c r="L4" s="1">
         <v>4842222</v>
       </c>
-      <c r="M4" s="3">
+      <c r="M4" s="1">
         <v>4842222</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N4" s="1">
+        <v>4842222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="1">
         <f>12740617+4000000</f>
         <v>16740617</v>
       </c>
-      <c r="C5" s="3">
+      <c r="D5" s="1">
         <v>15256287.900000002</v>
       </c>
-      <c r="D5" s="3">
+      <c r="E5" s="1">
         <v>15653414.699999999</v>
       </c>
-      <c r="E5" s="3">
+      <c r="F5" s="1">
         <v>16580043.899999999</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="3">
         <v>17903799.900000002</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="1">
         <v>18102363.300000001</v>
       </c>
-      <c r="H5" s="3">
+      <c r="I5" s="1">
         <v>19591588.800000001</v>
       </c>
-      <c r="I5" s="3">
+      <c r="J5" s="1">
         <v>19955621.699999999</v>
       </c>
-      <c r="J5" s="3">
+      <c r="K5" s="1">
         <v>21941255.699999999</v>
       </c>
-      <c r="K5" s="3">
+      <c r="L5" s="1">
         <v>23629044.599999998</v>
       </c>
-      <c r="L5" s="3">
+      <c r="M5" s="1">
         <v>24522579.899999999</v>
       </c>
-      <c r="M5" s="3">
+      <c r="N5" s="1">
         <v>24787331.099999998</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="1">
         <v>15500000</v>
       </c>
-      <c r="C6" s="3">
+      <c r="D6" s="1">
         <v>14153718</v>
       </c>
-      <c r="D6" s="3">
+      <c r="E6" s="1">
         <v>13961718</v>
       </c>
-      <c r="E6" s="3">
+      <c r="F6" s="1">
         <v>14057718</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="3">
         <v>14249718</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H6" s="1">
         <v>14537718</v>
       </c>
-      <c r="H6" s="3">
+      <c r="I6" s="1">
         <v>14537718</v>
       </c>
-      <c r="I6" s="3">
+      <c r="J6" s="1">
         <v>14537718</v>
       </c>
-      <c r="J6" s="3">
+      <c r="K6" s="1">
         <v>14537718</v>
       </c>
-      <c r="K6" s="3">
+      <c r="L6" s="1">
         <v>14537718</v>
       </c>
-      <c r="L6" s="3">
+      <c r="M6" s="1">
         <v>14537718</v>
       </c>
-      <c r="M6" s="3">
+      <c r="N6" s="1">
         <v>14537718</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="1">
         <v>1615000</v>
       </c>
-      <c r="C7" s="3">
+      <c r="D7" s="1">
         <v>1615000</v>
       </c>
-      <c r="D7" s="3">
+      <c r="E7" s="1">
         <v>1615000</v>
       </c>
-      <c r="E7" s="3">
-        <v>1615000</v>
-      </c>
-      <c r="F7" s="3">
+      <c r="F7" s="1">
         <v>1615000</v>
       </c>
       <c r="G7" s="3">
         <v>1615000</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="1">
         <v>1615000</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="1">
         <v>1615000</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7" s="1">
         <v>1615000</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7" s="1">
         <v>1615000</v>
       </c>
-      <c r="L7" s="3">
+      <c r="L7" s="1">
         <v>1615000</v>
       </c>
-      <c r="M7" s="3">
+      <c r="M7" s="1">
         <v>1615000</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N7" s="1">
+        <v>1615000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="1">
         <v>5007183</v>
       </c>
-      <c r="C8" s="3">
+      <c r="D8" s="1">
         <v>5818955.5</v>
       </c>
-      <c r="D8" s="3">
+      <c r="E8" s="1">
         <v>6904268.91764706</v>
       </c>
-      <c r="E8" s="3">
+      <c r="F8" s="1">
         <v>6994249.7176470589</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G8" s="3">
         <v>7338063.717647058</v>
       </c>
-      <c r="G8" s="3">
+      <c r="H8" s="1">
         <v>8099460.3176470604</v>
       </c>
-      <c r="H8" s="3">
+      <c r="I8" s="1">
         <v>7980649.8176470585</v>
       </c>
-      <c r="I8" s="3">
+      <c r="J8" s="1">
         <v>8814764.41764706</v>
       </c>
-      <c r="J8" s="3">
+      <c r="K8" s="1">
         <v>9905482.91764706</v>
       </c>
-      <c r="K8" s="3">
+      <c r="L8" s="1">
         <v>9636004.0176470578</v>
       </c>
-      <c r="L8" s="3">
+      <c r="M8" s="1">
         <v>10504541.217647059</v>
       </c>
-      <c r="M8" s="3">
+      <c r="N8" s="1">
         <v>10997612.517647058</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1">
         <v>4500000</v>
       </c>
-      <c r="C9" s="3">
+      <c r="D9" s="1">
         <v>4835636</v>
       </c>
-      <c r="D9" s="3">
+      <c r="E9" s="1">
         <v>4787636</v>
       </c>
-      <c r="E9" s="3">
+      <c r="F9" s="1">
         <v>4787636</v>
       </c>
-      <c r="F9" s="3">
+      <c r="G9" s="3">
         <v>4859636</v>
       </c>
-      <c r="G9" s="3">
+      <c r="H9" s="1">
         <v>4931636</v>
       </c>
-      <c r="H9" s="3">
+      <c r="I9" s="1">
         <v>4931636</v>
       </c>
-      <c r="I9" s="3">
+      <c r="J9" s="1">
         <v>4931636</v>
       </c>
-      <c r="J9" s="3">
+      <c r="K9" s="1">
         <v>4931636</v>
       </c>
-      <c r="K9" s="3">
+      <c r="L9" s="1">
         <v>4931636</v>
       </c>
-      <c r="L9" s="3">
+      <c r="M9" s="1">
         <v>4931636</v>
       </c>
-      <c r="M9" s="3">
+      <c r="N9" s="1">
         <v>4931636</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="1">
         <v>1690657</v>
       </c>
-      <c r="C10" s="3">
+      <c r="D10" s="1">
         <v>1690000</v>
       </c>
-      <c r="D10" s="3">
+      <c r="E10" s="1">
         <v>1690000</v>
       </c>
-      <c r="E10" s="3">
-        <v>1690000</v>
-      </c>
-      <c r="F10" s="3">
+      <c r="F10" s="1">
         <v>1690000</v>
       </c>
       <c r="G10" s="3">
         <v>1690000</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="1">
         <v>1690000</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="1">
         <v>1690000</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J10" s="1">
         <v>1690000</v>
       </c>
-      <c r="K10" s="3">
+      <c r="K10" s="1">
         <v>1690000</v>
       </c>
-      <c r="L10" s="3">
+      <c r="L10" s="1">
         <v>1690000</v>
       </c>
-      <c r="M10" s="3">
+      <c r="M10" s="1">
         <v>1690000</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N10" s="1">
+        <v>1690000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="1">
         <v>3500000</v>
       </c>
-      <c r="C11" s="3">
+      <c r="D11" s="1">
         <v>1100000</v>
       </c>
-      <c r="D11" s="3">
+      <c r="E11" s="1">
         <v>1400000</v>
       </c>
-      <c r="E11" s="3">
-        <v>1400000</v>
-      </c>
-      <c r="F11" s="3">
+      <c r="F11" s="1">
         <v>1400000</v>
       </c>
       <c r="G11" s="3">
         <v>1400000</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="1">
         <v>1400000</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="1">
         <v>1400000</v>
       </c>
-      <c r="J11" s="3">
+      <c r="J11" s="1">
         <v>1400000</v>
       </c>
-      <c r="K11" s="3">
+      <c r="K11" s="1">
         <v>1400000</v>
       </c>
-      <c r="L11" s="3">
+      <c r="L11" s="1">
         <v>1400000</v>
       </c>
-      <c r="M11" s="3">
+      <c r="M11" s="1">
         <v>1400000</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N11" s="1">
+        <v>1400000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="1">
         <v>1500000</v>
       </c>
-      <c r="C12" s="3">
+      <c r="D12" s="1">
         <v>1499369</v>
       </c>
-      <c r="D12" s="3">
+      <c r="E12" s="1">
         <v>1497398</v>
       </c>
-      <c r="E12" s="3">
+      <c r="F12" s="1">
         <v>1496587</v>
       </c>
-      <c r="F12" s="3">
+      <c r="G12" s="3">
         <v>1496277</v>
       </c>
-      <c r="G12" s="3">
+      <c r="H12" s="1">
         <v>1494945</v>
       </c>
-      <c r="H12" s="3">
+      <c r="I12" s="1">
         <v>1495471</v>
       </c>
-      <c r="I12" s="3">
+      <c r="J12" s="1">
         <v>1492850</v>
       </c>
-      <c r="J12" s="3">
+      <c r="K12" s="1">
         <v>1491623</v>
       </c>
-      <c r="K12" s="3">
+      <c r="L12" s="1">
         <v>1491916</v>
       </c>
-      <c r="L12" s="3">
+      <c r="M12" s="1">
         <v>1491019</v>
       </c>
-      <c r="M12" s="3">
+      <c r="N12" s="1">
         <v>1489802</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="1">
         <v>50000</v>
       </c>
-      <c r="C13" s="3">
+      <c r="D13" s="1">
         <v>211118</v>
       </c>
-      <c r="D13" s="3">
+      <c r="E13" s="1">
         <v>211118</v>
       </c>
-      <c r="E13" s="3">
-        <v>211118</v>
-      </c>
-      <c r="F13" s="3">
+      <c r="F13" s="1">
         <v>211118</v>
       </c>
       <c r="G13" s="3">
         <v>211118</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="1">
         <v>211118</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="1">
         <v>211118</v>
       </c>
-      <c r="J13" s="3">
+      <c r="J13" s="1">
         <v>211118</v>
       </c>
-      <c r="K13" s="3">
+      <c r="K13" s="1">
         <v>211118</v>
       </c>
-      <c r="L13" s="3">
+      <c r="L13" s="1">
         <v>211118</v>
       </c>
-      <c r="M13" s="3">
+      <c r="M13" s="1">
         <v>211118</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N13" s="1">
+        <v>211118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="1">
-        <v>0</v>
-      </c>
-      <c r="C14" s="3">
-        <v>0</v>
-      </c>
-      <c r="D14" s="3">
-        <v>0</v>
-      </c>
-      <c r="E14" s="3">
-        <v>0</v>
-      </c>
-      <c r="F14" s="3">
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0</v>
+      </c>
+      <c r="F14" s="1">
         <v>0</v>
       </c>
       <c r="G14" s="3">
         <v>0</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1">
         <v>2500000</v>
       </c>
-      <c r="I14" s="3">
-        <v>0</v>
-      </c>
-      <c r="J14" s="3">
-        <v>0</v>
-      </c>
-      <c r="K14" s="3">
-        <v>0</v>
-      </c>
-      <c r="L14" s="3">
-        <v>0</v>
-      </c>
-      <c r="M14" s="3">
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1">
+        <v>0</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
+      <c r="N14" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>